<commit_message>
update form surat cuti
</commit_message>
<xml_diff>
--- a/data_pegawai.xlsx
+++ b/data_pegawai.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Digitalisasi\Downloads\DataCuti\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DataCuti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74D03EA3-591B-4B13-A1B1-1C3ABCFBB3E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51E9B0B4-5BB2-4720-8784-FCE6B38159BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="185">
   <si>
     <t>NO</t>
   </si>
@@ -349,6 +349,246 @@
   </si>
   <si>
     <t>Penata Muda Tingkat I, III/b</t>
+  </si>
+  <si>
+    <t>CONTACT</t>
+  </si>
+  <si>
+    <t>+62 812-7183-3370</t>
+  </si>
+  <si>
+    <t>+62 813-6798-4971</t>
+  </si>
+  <si>
+    <t>+62 859-3353-2713</t>
+  </si>
+  <si>
+    <t>+62 812-3428-4752</t>
+  </si>
+  <si>
+    <t>+62 813-6601-7078</t>
+  </si>
+  <si>
+    <t>+62 822-8126-9317</t>
+  </si>
+  <si>
+    <t>+62 812-9379-3947</t>
+  </si>
+  <si>
+    <t>+62 882-7424-0921</t>
+  </si>
+  <si>
+    <t>+62 831-4490-2607</t>
+  </si>
+  <si>
+    <t>+62 813-7959-9269</t>
+  </si>
+  <si>
+    <t>+62 813-7387-1076</t>
+  </si>
+  <si>
+    <t>+62 838-0269-2022</t>
+  </si>
+  <si>
+    <t>+62 852-6796-8380</t>
+  </si>
+  <si>
+    <t>+62 882-7641-6419</t>
+  </si>
+  <si>
+    <t>+62 852-6851-1882</t>
+  </si>
+  <si>
+    <t>+62 813-6703-3099</t>
+  </si>
+  <si>
+    <t>+62 813-1132-3381</t>
+  </si>
+  <si>
+    <t>+62 819-4740-0861</t>
+  </si>
+  <si>
+    <t>+62 813-7341-4313</t>
+  </si>
+  <si>
+    <t>+62 822-7809-3771</t>
+  </si>
+  <si>
+    <t>+62 852-7323-3705</t>
+  </si>
+  <si>
+    <t>+62 838-0238-5374</t>
+  </si>
+  <si>
+    <t>+62 852-7367-5324</t>
+  </si>
+  <si>
+    <t>+62 815-3939-6003</t>
+  </si>
+  <si>
+    <t>+62 812-7327-4662</t>
+  </si>
+  <si>
+    <t>+62 852-9349-3394</t>
+  </si>
+  <si>
+    <t>+62 813-6710-8434</t>
+  </si>
+  <si>
+    <t>+62 813-2876-7144</t>
+  </si>
+  <si>
+    <t>+62 852-7369-7604</t>
+  </si>
+  <si>
+    <t>+62 852-6609-8967</t>
+  </si>
+  <si>
+    <t>+62 852-6377-7754</t>
+  </si>
+  <si>
+    <t>+62 821-7528-8582</t>
+  </si>
+  <si>
+    <t>+62 852-7479-7555</t>
+  </si>
+  <si>
+    <t>+62 813-6891-9717</t>
+  </si>
+  <si>
+    <t>+62 812-6378-7087</t>
+  </si>
+  <si>
+    <t>+62 858-3242-3623</t>
+  </si>
+  <si>
+    <t>+62 821-8442-4051</t>
+  </si>
+  <si>
+    <t>+62 819-4925-8505</t>
+  </si>
+  <si>
+    <t>+62 813-6769-3118</t>
+  </si>
+  <si>
+    <t>+62 852-6334-0902</t>
+  </si>
+  <si>
+    <t>+62 821-7809-9007</t>
+  </si>
+  <si>
+    <t>Jelutung</t>
+  </si>
+  <si>
+    <t>Jl. Taman Siswa Rt 009</t>
+  </si>
+  <si>
+    <t>Payung</t>
+  </si>
+  <si>
+    <t>Jl. Tengah</t>
+  </si>
+  <si>
+    <t>Berok</t>
+  </si>
+  <si>
+    <t>Dusun Rambat</t>
+  </si>
+  <si>
+    <t>Jl. Pamekasan  Rt 2 Rw 2</t>
+  </si>
+  <si>
+    <t>Jl. Trans 1 Kurau Timur Rt.009</t>
+  </si>
+  <si>
+    <t>Jl. Teladan</t>
+  </si>
+  <si>
+    <t>Jl. Raya Koba, Desa Terentang</t>
+  </si>
+  <si>
+    <t>Jl. Raya Koba Km. 42</t>
+  </si>
+  <si>
+    <t>Gg. Mutiara Iii Girimaya</t>
+  </si>
+  <si>
+    <t>Jl. Widuri Bulan</t>
+  </si>
+  <si>
+    <t>Jl. Mesjid Nurul Falah</t>
+  </si>
+  <si>
+    <t>Gg. Tower Rt 06 Simpang Perlang</t>
+  </si>
+  <si>
+    <t>Jl. Hundani Lt. Pancur Pangkalan Balam Pangkalpinang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jl. Mesjid Dalam Rt 06 </t>
+  </si>
+  <si>
+    <t>Jl. Tiram Raya No 46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perumahan Tanjung Bunga </t>
+  </si>
+  <si>
+    <t>Jl. Adyaksa No. 180</t>
+  </si>
+  <si>
+    <t>Gang Haji</t>
+  </si>
+  <si>
+    <t>Jl. Sekolah</t>
+  </si>
+  <si>
+    <t>Jl. Depati Amir No.159, Rt.007</t>
+  </si>
+  <si>
+    <t>Jl. Jongkong No. 38</t>
+  </si>
+  <si>
+    <t>Gg. Merpati Ii No 035</t>
+  </si>
+  <si>
+    <t>Jl. Batin Tikal</t>
+  </si>
+  <si>
+    <t>Komp. Perumahan Guru Berok Koba</t>
+  </si>
+  <si>
+    <t>Jl. Komplek Guru Ii No 40</t>
+  </si>
+  <si>
+    <t>Koba</t>
+  </si>
+  <si>
+    <t>H.M Nur</t>
+  </si>
+  <si>
+    <t>Jl. Abdus Somad</t>
+  </si>
+  <si>
+    <t>Penyak</t>
+  </si>
+  <si>
+    <t>Jl. Kamboja Rt 005 Rw 002</t>
+  </si>
+  <si>
+    <t>Komplek Perumahan Guru No.34</t>
+  </si>
+  <si>
+    <t>Tangsi Lama</t>
+  </si>
+  <si>
+    <t>Jl. Sinar Surya Gg. Aster 1</t>
+  </si>
+  <si>
+    <t>ALAMAT</t>
+  </si>
+  <si>
+    <t>Jl. Fatmawati Kampak Gg. H. Bakier Graha Pinang Mas 1</t>
   </si>
 </sst>
 </file>
@@ -722,7 +962,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -731,9 +971,11 @@
     <col min="4" max="4" width="8" customWidth="1"/>
     <col min="5" max="5" width="42.6328125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="42.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="47.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -752,8 +994,14 @@
       <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G1" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -772,36 +1020,48 @@
       <c r="F2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>56</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>55</v>
       </c>
       <c r="D3" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="F3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+      <c r="G3" t="s">
+        <v>127</v>
+      </c>
+      <c r="H3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D4" t="s">
         <v>7</v>
@@ -812,36 +1072,48 @@
       <c r="F4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G4" t="s">
+        <v>107</v>
+      </c>
+      <c r="H4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>93</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>92</v>
       </c>
       <c r="D5" t="s">
-        <v>7</v>
+        <v>90</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="F5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+        <v>91</v>
+      </c>
+      <c r="G5" t="s">
+        <v>144</v>
+      </c>
+      <c r="H5" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D6" t="s">
         <v>7</v>
@@ -852,16 +1124,22 @@
       <c r="F6" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G6" t="s">
+        <v>108</v>
+      </c>
+      <c r="H6" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D7" t="s">
         <v>7</v>
@@ -872,16 +1150,22 @@
       <c r="F7" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H7" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s">
         <v>7</v>
@@ -892,16 +1176,22 @@
       <c r="F8" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G8" t="s">
+        <v>114</v>
+      </c>
+      <c r="H8" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D9" t="s">
         <v>7</v>
@@ -912,36 +1202,48 @@
       <c r="F9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H9" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>95</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="D10" t="s">
-        <v>7</v>
+        <v>90</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="F10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+        <v>91</v>
+      </c>
+      <c r="G10" t="s">
+        <v>145</v>
+      </c>
+      <c r="H10" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C11" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="D11" t="s">
         <v>7</v>
@@ -952,16 +1254,22 @@
       <c r="F11" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G11" t="s">
+        <v>111</v>
+      </c>
+      <c r="H11" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="C12" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="D12" t="s">
         <v>7</v>
@@ -972,36 +1280,48 @@
       <c r="F12" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G12" t="s">
+        <v>112</v>
+      </c>
+      <c r="H12" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>82</v>
       </c>
       <c r="C13" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="D13" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="F13" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+      <c r="G13" t="s">
+        <v>140</v>
+      </c>
+      <c r="H13" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C14" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="D14" t="s">
         <v>7</v>
@@ -1012,76 +1332,100 @@
       <c r="F14" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G14" t="s">
+        <v>113</v>
+      </c>
+      <c r="H14" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>34</v>
+        <v>66</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="D15" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="F15" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+      <c r="G15" t="s">
+        <v>132</v>
+      </c>
+      <c r="H15" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>80</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>79</v>
       </c>
       <c r="D16" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="E16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F16" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+      <c r="G16" t="s">
+        <v>139</v>
+      </c>
+      <c r="H16" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="C17" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="D17" t="s">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="E17" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F17" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+      <c r="G17" t="s">
+        <v>115</v>
+      </c>
+      <c r="H17" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D18" t="s">
         <v>41</v>
@@ -1092,216 +1436,279 @@
       <c r="F18" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G18" t="s">
+        <v>123</v>
+      </c>
+      <c r="H18" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="C19" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="D19" t="s">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="E19" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F19" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+      <c r="G19" t="s">
+        <v>116</v>
+      </c>
+      <c r="H19" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>48</v>
+        <v>76</v>
       </c>
       <c r="C20" t="s">
-        <v>47</v>
+        <v>75</v>
       </c>
       <c r="D20" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="E20" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F20" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+      <c r="G20" t="s">
+        <v>137</v>
+      </c>
+      <c r="H20" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="C21" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="D21" t="s">
-        <v>51</v>
+        <v>7</v>
       </c>
       <c r="E21" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F21" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+      <c r="G21" t="s">
+        <v>117</v>
+      </c>
+      <c r="H21" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="C22" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="D22" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="E22" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F22" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+      <c r="G22" t="s">
+        <v>122</v>
+      </c>
+      <c r="H22" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="C23" t="s">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="D23" t="s">
-        <v>51</v>
+        <v>7</v>
       </c>
       <c r="E23" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F23" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+      <c r="G23" t="s">
+        <v>118</v>
+      </c>
+      <c r="H23" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="C24" t="s">
-        <v>57</v>
+        <v>88</v>
       </c>
       <c r="D24" t="s">
-        <v>51</v>
+        <v>90</v>
       </c>
       <c r="E24" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F24" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+        <v>91</v>
+      </c>
+      <c r="G24" t="s">
+        <v>143</v>
+      </c>
+      <c r="H24" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="C25" t="s">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="D25" t="s">
-        <v>51</v>
+        <v>7</v>
       </c>
       <c r="E25" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F25" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+      <c r="G25" t="s">
+        <v>119</v>
+      </c>
+      <c r="H25" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="C26" t="s">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="D26" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="E26" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F26" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+      <c r="G26" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="C27" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="D27" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="E27" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F27" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+      <c r="G27" t="s">
+        <v>124</v>
+      </c>
+      <c r="H27" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>66</v>
+        <v>40</v>
       </c>
       <c r="C28" t="s">
-        <v>65</v>
+        <v>39</v>
       </c>
       <c r="D28" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="E28" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F28" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+      <c r="G28" t="s">
+        <v>121</v>
+      </c>
+      <c r="H28" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C29" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D29" t="s">
         <v>51</v>
@@ -1312,16 +1719,22 @@
       <c r="F29" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G29" t="s">
+        <v>134</v>
+      </c>
+      <c r="H29" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="C30" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="D30" t="s">
         <v>51</v>
@@ -1332,16 +1745,22 @@
       <c r="F30" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G30" t="s">
+        <v>125</v>
+      </c>
+      <c r="H30" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="C31" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="D31" t="s">
         <v>51</v>
@@ -1352,16 +1771,22 @@
       <c r="F31" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G31" t="s">
+        <v>141</v>
+      </c>
+      <c r="H31" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="C32" t="s">
-        <v>73</v>
+        <v>53</v>
       </c>
       <c r="D32" t="s">
         <v>51</v>
@@ -1372,16 +1797,22 @@
       <c r="F32" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G32" t="s">
+        <v>126</v>
+      </c>
+      <c r="H32" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="C33" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="D33" t="s">
         <v>51</v>
@@ -1392,16 +1823,22 @@
       <c r="F33" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G33" t="s">
+        <v>133</v>
+      </c>
+      <c r="H33" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="C34" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="D34" t="s">
         <v>51</v>
@@ -1412,16 +1849,22 @@
       <c r="F34" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G34" t="s">
+        <v>128</v>
+      </c>
+      <c r="H34" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C35" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="D35" t="s">
         <v>51</v>
@@ -1432,16 +1875,22 @@
       <c r="F35" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G35" t="s">
+        <v>129</v>
+      </c>
+      <c r="H35" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="C36" t="s">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="D36" t="s">
         <v>51</v>
@@ -1452,16 +1901,22 @@
       <c r="F36" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G36" t="s">
+        <v>130</v>
+      </c>
+      <c r="H36" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C37" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="D37" t="s">
         <v>51</v>
@@ -1472,16 +1927,22 @@
       <c r="F37" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G37" t="s">
+        <v>138</v>
+      </c>
+      <c r="H37" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>86</v>
+        <v>64</v>
       </c>
       <c r="C38" t="s">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="D38" t="s">
         <v>51</v>
@@ -1490,70 +1951,91 @@
         <v>103</v>
       </c>
       <c r="F38" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+      <c r="G38" t="s">
+        <v>131</v>
+      </c>
+      <c r="H38" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="C39" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="D39" t="s">
-        <v>90</v>
+        <v>51</v>
       </c>
       <c r="E39" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F39" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+      <c r="G39" t="s">
+        <v>135</v>
+      </c>
+      <c r="H39" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="C40" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="D40" t="s">
-        <v>90</v>
+        <v>51</v>
       </c>
       <c r="E40" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F40" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+      <c r="G40" t="s">
+        <v>136</v>
+      </c>
+      <c r="H40" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="C41" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="D41" t="s">
-        <v>90</v>
+        <v>51</v>
       </c>
       <c r="E41" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F41" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+        <v>87</v>
+      </c>
+      <c r="G41" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1571,6 +2053,9 @@
       </c>
       <c r="F42" t="s">
         <v>98</v>
+      </c>
+      <c r="G42" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>